<commit_message>
Remove mission from purposes (Option C)
- schema.ts: removed mission column from purposes table
- storage.ts: removed mission TEXT from CREATE TABLE, commented out migration
- xlsx-io.ts: removed mission from export, import, and SHEET_COLUMNS
- generate-template.cjs: removed mission column from Purposes sheet
- wizard.tsx: stripped PrincipleCard/Mission Cards UI, simplified to Purpose-only
- dashboard.tsx: updated nudge text from 'Purpose & Mission' to 'Purpose'
- Regenerated XLSX template

Immutable Laws (per puzzle piece) now handle all boundary-setting that
mission previously served.
</commit_message>
<xml_diff>
--- a/server/templates/unpuzzle-life-template.xlsx
+++ b/server/templates/unpuzzle-life-template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="251">
   <si>
     <t>UnPuzzle Life — Data Workbook</t>
   </si>
@@ -50,7 +50,7 @@
     <t>Purposes</t>
   </si>
   <si>
-    <t>Life purpose statements and mission</t>
+    <t>Life purpose statements</t>
   </si>
   <si>
     <t>statement</t>
@@ -191,58 +191,52 @@
     <t>None</t>
   </si>
   <si>
-    <t>mission</t>
-  </si>
-  <si>
     <t>Your purpose statement (e.g. 'To live with intention and serve others')</t>
   </si>
   <si>
-    <t>Mission statement</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
+    <t>puzzle_piece</t>
+  </si>
+  <si>
+    <t>vision_text</t>
+  </si>
+  <si>
+    <t>icon</t>
+  </si>
+  <si>
+    <t>sort_order</t>
+  </si>
+  <si>
+    <t>archived</t>
+  </si>
+  <si>
+    <t>archived_at</t>
+  </si>
+  <si>
+    <t>Area name (e.g. 'Morning Routine', 'Career Growth')</t>
+  </si>
+  <si>
+    <t>reason | finance | fitness | talent | pleasure</t>
+  </si>
+  <si>
+    <t>Your immersive area vision text</t>
+  </si>
+  <si>
+    <t>Lucide icon name</t>
+  </si>
+  <si>
+    <t>Display order (number)</t>
+  </si>
+  <si>
+    <t>0 = active, 1 = archived</t>
+  </si>
+  <si>
+    <t>Archive timestamp (ISO 8601)</t>
+  </si>
+  <si>
     <t>No</t>
-  </si>
-  <si>
-    <t>puzzle_piece</t>
-  </si>
-  <si>
-    <t>vision_text</t>
-  </si>
-  <si>
-    <t>icon</t>
-  </si>
-  <si>
-    <t>sort_order</t>
-  </si>
-  <si>
-    <t>archived</t>
-  </si>
-  <si>
-    <t>archived_at</t>
-  </si>
-  <si>
-    <t>Area name (e.g. 'Morning Routine', 'Career Growth')</t>
-  </si>
-  <si>
-    <t>reason | finance | fitness | talent | pleasure</t>
-  </si>
-  <si>
-    <t>Your immersive area vision text</t>
-  </si>
-  <si>
-    <t>Lucide icon name</t>
-  </si>
-  <si>
-    <t>Display order (number)</t>
-  </si>
-  <si>
-    <t>0 = active, 1 = archived</t>
-  </si>
-  <si>
-    <t>Archive timestamp (ISO 8601)</t>
   </si>
   <si>
     <t>area_name</t>
@@ -1542,77 +1536,77 @@
         <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>150</v>
-      </c>
       <c r="H1" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>157</v>
-      </c>
       <c r="H2" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1639,77 +1633,77 @@
         <v>35</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>168</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1740,143 +1734,143 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>179</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="M2" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>191</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1901,89 +1895,89 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>199</v>
-      </c>
       <c r="I1" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="G2" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>205</v>
-      </c>
       <c r="I2" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2012,125 +2006,125 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F1" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="K1" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>212</v>
-      </c>
       <c r="M1" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="K2" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>222</v>
-      </c>
       <c r="M2" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2157,98 +2151,98 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>227</v>
-      </c>
       <c r="J1" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>235</v>
-      </c>
       <c r="J2" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2273,89 +2267,89 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>239</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>246</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2376,35 +2370,35 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2415,35 +2409,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" ht="25" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="5" t="s">
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2469,68 +2453,68 @@
         <v>11</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2551,44 +2535,44 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2613,71 +2597,71 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>82</v>
-      </c>
       <c r="F1" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="D2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>86</v>
-      </c>
       <c r="F2" s="6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2706,122 +2690,122 @@
         <v>8</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>94</v>
-      </c>
       <c r="L1" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="J2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="L2" s="6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2847,143 +2831,143 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="K1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="J1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="K1" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>108</v>
-      </c>
       <c r="O1" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="L2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="M2" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="L2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>115</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -3005,44 +2989,44 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="D1" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3065,134 +3049,134 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="M1" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="J2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="J2" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="K2" s="6" t="s">
+      <c r="M2" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>144</v>
-      </c>
       <c r="N2" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 1: Schema & Backend Foundation (v2 rebuild)
- Add 8 new Drizzle tables: environmentPeople, environmentPlaces,
  environmentThings, projectEnvironment, responsibilities, roles,
  rolePeople, nonNegotiables
- Add status column (draft/project/routine/archived) to identities
- Add ~30 new IStorage interface methods with CRUD implementations
- Add REST API routes for all new entities
- Extend XLSX import/export with 6 new sheets
- Update template generator with new sheets and status column
- Include v2 spec document in docs/
</commit_message>
<xml_diff>
--- a/server/templates/unpuzzle-life-template.xlsx
+++ b/server/templates/unpuzzle-life-template.xlsx
@@ -20,14 +20,20 @@
     <sheet sheetId="14" name="Anti Habits" state="visible" r:id="rId17"/>
     <sheet sheetId="15" name="Immutable Laws" state="visible" r:id="rId18"/>
     <sheet sheetId="16" name="Immutable Law Logs" state="visible" r:id="rId19"/>
-    <sheet sheetId="17" name="Wizard State" state="visible" r:id="rId20"/>
+    <sheet sheetId="17" name="Environment People" state="visible" r:id="rId20"/>
+    <sheet sheetId="18" name="Environment Places" state="visible" r:id="rId21"/>
+    <sheet sheetId="19" name="Environment Things" state="visible" r:id="rId22"/>
+    <sheet sheetId="20" name="Responsibilities" state="visible" r:id="rId23"/>
+    <sheet sheetId="21" name="Roles" state="visible" r:id="rId24"/>
+    <sheet sheetId="22" name="Non Negotiables" state="visible" r:id="rId25"/>
+    <sheet sheetId="23" name="Wizard State" state="visible" r:id="rId26"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="292">
   <si>
     <t>UnPuzzle Life — Data Workbook</t>
   </si>
@@ -182,6 +188,45 @@
     <t>immutable_law_title, puzzle_piece, date, kept</t>
   </si>
   <si>
+    <t>Environment People</t>
+  </si>
+  <si>
+    <t>Shared people entities (born in projects, reused in roles)</t>
+  </si>
+  <si>
+    <t>Environment Places</t>
+  </si>
+  <si>
+    <t>Shared places entities (born in projects, reused in responsibilities)</t>
+  </si>
+  <si>
+    <t>Environment Things</t>
+  </si>
+  <si>
+    <t>Shared things entities (born in projects, reused in responsibilities)</t>
+  </si>
+  <si>
+    <t>Responsibilities</t>
+  </si>
+  <si>
+    <t>Recurring chores and life maintenance tasks</t>
+  </si>
+  <si>
+    <t>Roles</t>
+  </si>
+  <si>
+    <t>Recurring commitments to specific people or groups</t>
+  </si>
+  <si>
+    <t>Non Negotiables</t>
+  </si>
+  <si>
+    <t>Two-layer boundaries: global (per puzzle piece) and area-specific</t>
+  </si>
+  <si>
+    <t>puzzle_piece, statement</t>
+  </si>
+  <si>
     <t>Wizard State</t>
   </si>
   <si>
@@ -308,6 +353,9 @@
     <t>location</t>
   </si>
   <si>
+    <t>status</t>
+  </si>
+  <si>
     <t>Identity statement (e.g. 'I am a person who exercises daily')</t>
   </si>
   <si>
@@ -335,6 +383,9 @@
     <t>Where this takes place</t>
   </si>
   <si>
+    <t>draft | project | routine</t>
+  </si>
+  <si>
     <t>time</t>
   </si>
   <si>
@@ -413,9 +464,6 @@
     <t>result</t>
   </si>
   <si>
-    <t>status</t>
-  </si>
-  <si>
     <t>recurrence</t>
   </si>
   <si>
@@ -768,6 +816,87 @@
   </si>
   <si>
     <t>Suggested anti-habit title</t>
+  </si>
+  <si>
+    <t>relationship</t>
+  </si>
+  <si>
+    <t>Person's name (e.g. 'Marcus')</t>
+  </si>
+  <si>
+    <t>Relationship (e.g. 'Son', 'Wife', 'Friend')</t>
+  </si>
+  <si>
+    <t>Place name (e.g. 'Master Bedroom')</t>
+  </si>
+  <si>
+    <t>room | vehicle | location</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>Thing name (e.g. '2019 Honda Accord')</t>
+  </si>
+  <si>
+    <t>vehicle | equipment | tool</t>
+  </si>
+  <si>
+    <t>cadence</t>
+  </si>
+  <si>
+    <t>day_of_week</t>
+  </si>
+  <si>
+    <t>custom_cron_expr</t>
+  </si>
+  <si>
+    <t>is_preset</t>
+  </si>
+  <si>
+    <t>Responsibility name (e.g. 'Bathroom', 'Laundry-Wash')</t>
+  </si>
+  <si>
+    <t>Linked place name (must match an Environment Place)</t>
+  </si>
+  <si>
+    <t>Linked thing name (must match an Environment Thing)</t>
+  </si>
+  <si>
+    <t>daily | weekly | biweekly | monthly | custom</t>
+  </si>
+  <si>
+    <t>Day of week (e.g. 'wednesday')</t>
+  </si>
+  <si>
+    <t>Custom cron expression for complex schedules</t>
+  </si>
+  <si>
+    <t>0 = user-created, 1 = preset</t>
+  </si>
+  <si>
+    <t>people_names</t>
+  </si>
+  <si>
+    <t>Role name (e.g. 'Help Marcus with homework')</t>
+  </si>
+  <si>
+    <t>Optional detail</t>
+  </si>
+  <si>
+    <t>daily | weekdays | weekly | biweekly | monthly | custom</t>
+  </si>
+  <si>
+    <t>Day of week</t>
+  </si>
+  <si>
+    <t>Linked people names, separated by semicolons</t>
+  </si>
+  <si>
+    <t>Non-negotiable boundary statement</t>
+  </si>
+  <si>
+    <t>Linked area name (empty = global boundary)</t>
   </si>
   <si>
     <t>current_phase</t>
@@ -1245,7 +1374,7 @@
   <sheetPr>
     <tabColor rgb="0D4F4F"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1502,9 +1631,93 @@
         <v>52</v>
       </c>
       <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="4">
+      <c r="B21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="4">
         <v>0</v>
       </c>
     </row>
@@ -1536,77 +1749,77 @@
         <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1633,77 +1846,77 @@
         <v>35</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1734,143 +1947,143 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1895,89 +2108,89 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2006,125 +2219,125 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2151,98 +2364,98 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2267,89 +2480,89 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2360,45 +2573,111 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>247</v>
+        <v>11</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="2" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>69</v>
+        <v>263</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="2" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="2" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2422,12 +2701,265 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="3" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2453,68 +2985,68 @@
         <v>11</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2535,44 +3067,44 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2597,71 +3129,71 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2672,7 +3204,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2681,131 +3213,140 @@
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="30" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="11" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" ht="25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>60</v>
+        <v>106</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" ht="35" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>67</v>
+        <v>116</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2831,143 +3372,143 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="J1" s="5" t="s">
+      <c r="N1" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="O1" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="F2" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="G2" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="J2" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>84</v>
-      </c>
       <c r="K2" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="L2" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="M2" s="6" t="s">
-        <v>99</v>
-      </c>
       <c r="N2" s="6" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2989,44 +3530,44 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -3049,134 +3590,134 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>